<commit_message>
fix: resolve timezone mismatch, wbs calculation, widget validation rollback, deduplication, and mobile layout
</commit_message>
<xml_diff>
--- a/docs/wbs/wbs_helpdesk_system.xlsx
+++ b/docs/wbs/wbs_helpdesk_system.xlsx
@@ -148,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -203,6 +203,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2162,15 +2165,14 @@
       <c r="E37" s="18" t="n"/>
       <c r="F37" s="18" t="n"/>
       <c r="G37" s="19">
-        <f>SUM(G6:G34)/2</f>
+        <f>SUM(G6,G9,G13,G17,G21,G25,G29,G33)</f>
         <v/>
       </c>
-      <c r="H37" s="17" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-      <c r="I37" s="20" t="inlineStr">
+      <c r="H37" s="20">
+        <f>SUM(H6,H9,H13,H17,H21,H25,H29,H33)</f>
+        <v/>
+      </c>
+      <c r="I37" s="21" t="inlineStr">
         <is>
           <t>Status: Siap Eksekusi (Ready)</t>
         </is>

</xml_diff>